<commit_message>
Update New Orleans expense report with Denver lunch and rebooking detail
Corrects airfare description to reflect the full round-trip fare and
the mechanical-delay rebooking through Denver; adds the $31.08 Great
Divide C lunch receipt from the layover.
</commit_message>
<xml_diff>
--- a/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
+++ b/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\Group-2\travel\trips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B26F4BB-075A-495D-8099-04520BC40BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D579A71-AF67-47A4-9961-D169BBD03062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35880" yWindow="2190" windowWidth="29040" windowHeight="17520" xr2:uid="{BDF1D293-00A6-47DF-A729-E60B3B82F4CB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{665F24CF-46C1-42D5-94C2-B96555D6B5FA}"/>
   </bookViews>
   <sheets>
     <sheet name="ER Detail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
   <si>
     <t>UNIFOCUS EXPENSE REPORT  |  New Orleans - InterContinental (HM Alpha)</t>
   </si>
@@ -90,7 +90,7 @@
     <t>PERSONAL</t>
   </si>
   <si>
-    <t>SW OMA-DAL-MSY (CVMCLW) - card charge portion, Visa -2674</t>
+    <t>SW round-trip OMA-MSY (CVMCLW): outbound OMA-DEN-MSY (WN2060/WN1643, rebooked from OMA-DAL-MSY - mechanical delay); return MSY-STL-OMA 7/9 (WN3021/WN4912) - card charge portion, Visa -2674</t>
   </si>
   <si>
     <t>Air Fare</t>
@@ -102,7 +102,13 @@
     <t/>
   </si>
   <si>
-    <t>SW OMA-DAL-MSY (CVMCLW) - SW travel credit applied</t>
+    <t>SW round-trip OMA-MSY (CVMCLW) - SW travel credit applied</t>
+  </si>
+  <si>
+    <t>HMSHost/Great Divide C, Denver Airport (DEN layover, mechanical delay) - taco barbacoa, soda, tip</t>
+  </si>
+  <si>
+    <t>Lunch</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -318,10 +324,10 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -660,11 +666,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{702BFB93-BC25-4CED-B8CD-CD389FA6A731}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD4AD5B1-FA26-448F-B874-DC9BF431DEC5}">
   <sheetPr>
     <tabColor rgb="FFB6752E"/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" customWidth="1"/>
@@ -814,24 +820,38 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="7"/>
+      <c r="A7" s="7">
+        <v>46209</v>
+      </c>
       <c r="B7" s="8" t="str">
-        <f>IF(A7="","",TEXT(A7,"ddd"))</f>
-        <v/>
-      </c>
-      <c r="C7" s="19"/>
+        <f>TEXT(A7,"ddd")</f>
+        <v>Mon</v>
+      </c>
+      <c r="C7" s="9">
+        <v>31.08</v>
+      </c>
       <c r="D7" s="10">
         <v>1</v>
       </c>
       <c r="E7" s="9">
         <f>C7*D7</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="20"/>
+        <v>31.08</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="13"/>
@@ -839,7 +859,7 @@
         <f>IF(A8="","",TEXT(A8,"ddd"))</f>
         <v/>
       </c>
-      <c r="C8" s="21"/>
+      <c r="C8" s="19"/>
       <c r="D8" s="16">
         <v>1</v>
       </c>
@@ -851,7 +871,7 @@
       <c r="G8" s="17"/>
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
-      <c r="J8" s="22"/>
+      <c r="J8" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="7"/>
@@ -859,7 +879,7 @@
         <f>IF(A9="","",TEXT(A9,"ddd"))</f>
         <v/>
       </c>
-      <c r="C9" s="19"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="10">
         <v>1</v>
       </c>
@@ -871,7 +891,7 @@
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
-      <c r="J9" s="20"/>
+      <c r="J9" s="22"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="13"/>
@@ -879,7 +899,7 @@
         <f>IF(A10="","",TEXT(A10,"ddd"))</f>
         <v/>
       </c>
-      <c r="C10" s="21"/>
+      <c r="C10" s="19"/>
       <c r="D10" s="16">
         <v>1</v>
       </c>
@@ -891,7 +911,7 @@
       <c r="G10" s="17"/>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
-      <c r="J10" s="22"/>
+      <c r="J10" s="20"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="7"/>
@@ -899,7 +919,7 @@
         <f>IF(A11="","",TEXT(A11,"ddd"))</f>
         <v/>
       </c>
-      <c r="C11" s="19"/>
+      <c r="C11" s="21"/>
       <c r="D11" s="10">
         <v>1</v>
       </c>
@@ -911,7 +931,7 @@
       <c r="G11" s="11"/>
       <c r="H11" s="11"/>
       <c r="I11" s="11"/>
-      <c r="J11" s="20"/>
+      <c r="J11" s="22"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="13"/>
@@ -919,7 +939,7 @@
         <f>IF(A12="","",TEXT(A12,"ddd"))</f>
         <v/>
       </c>
-      <c r="C12" s="21"/>
+      <c r="C12" s="19"/>
       <c r="D12" s="16">
         <v>1</v>
       </c>
@@ -931,7 +951,7 @@
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
-      <c r="J12" s="22"/>
+      <c r="J12" s="20"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="7"/>
@@ -939,7 +959,7 @@
         <f>IF(A13="","",TEXT(A13,"ddd"))</f>
         <v/>
       </c>
-      <c r="C13" s="19"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="10">
         <v>1</v>
       </c>
@@ -951,7 +971,7 @@
       <c r="G13" s="11"/>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
-      <c r="J13" s="20"/>
+      <c r="J13" s="22"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="13"/>
@@ -959,7 +979,7 @@
         <f>IF(A14="","",TEXT(A14,"ddd"))</f>
         <v/>
       </c>
-      <c r="C14" s="21"/>
+      <c r="C14" s="19"/>
       <c r="D14" s="16">
         <v>1</v>
       </c>
@@ -971,7 +991,7 @@
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
-      <c r="J14" s="22"/>
+      <c r="J14" s="20"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="7"/>
@@ -979,7 +999,7 @@
         <f>IF(A15="","",TEXT(A15,"ddd"))</f>
         <v/>
       </c>
-      <c r="C15" s="19"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="10">
         <v>1</v>
       </c>
@@ -991,7 +1011,7 @@
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
-      <c r="J15" s="20"/>
+      <c r="J15" s="22"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="13"/>
@@ -999,7 +1019,7 @@
         <f>IF(A16="","",TEXT(A16,"ddd"))</f>
         <v/>
       </c>
-      <c r="C16" s="21"/>
+      <c r="C16" s="19"/>
       <c r="D16" s="16">
         <v>1</v>
       </c>
@@ -1011,7 +1031,7 @@
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
-      <c r="J16" s="22"/>
+      <c r="J16" s="20"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="7"/>
@@ -1019,7 +1039,7 @@
         <f>IF(A17="","",TEXT(A17,"ddd"))</f>
         <v/>
       </c>
-      <c r="C17" s="19"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="10">
         <v>1</v>
       </c>
@@ -1031,7 +1051,7 @@
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
-      <c r="J17" s="20"/>
+      <c r="J17" s="22"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="13"/>
@@ -1039,7 +1059,7 @@
         <f>IF(A18="","",TEXT(A18,"ddd"))</f>
         <v/>
       </c>
-      <c r="C18" s="21"/>
+      <c r="C18" s="19"/>
       <c r="D18" s="16">
         <v>1</v>
       </c>
@@ -1051,7 +1071,7 @@
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
-      <c r="J18" s="22"/>
+      <c r="J18" s="20"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="7"/>
@@ -1059,7 +1079,7 @@
         <f>IF(A19="","",TEXT(A19,"ddd"))</f>
         <v/>
       </c>
-      <c r="C19" s="19"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="10">
         <v>1</v>
       </c>
@@ -1071,7 +1091,7 @@
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
-      <c r="J19" s="20"/>
+      <c r="J19" s="22"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="13"/>
@@ -1079,7 +1099,7 @@
         <f>IF(A20="","",TEXT(A20,"ddd"))</f>
         <v/>
       </c>
-      <c r="C20" s="21"/>
+      <c r="C20" s="19"/>
       <c r="D20" s="16">
         <v>1</v>
       </c>
@@ -1091,34 +1111,54 @@
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="22"/>
+      <c r="J20" s="20"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21" s="25">
-        <f>SUM(E5:E20)</f>
-        <v>861.3900000000001</v>
-      </c>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="23"/>
-      <c r="J21" s="23"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="8" t="str">
+        <f>IF(A21="","",TEXT(A21,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="C21" s="21"/>
+      <c r="D21" s="10">
+        <v>1</v>
+      </c>
+      <c r="E21" s="9">
+        <f>C21*D21</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="22"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" s="23"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="25">
+        <f>SUM(E5:E21)</f>
+        <v>892.47000000000014</v>
+      </c>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F20" xr:uid="{2C944181-E45B-4CC1-9968-F0DF99C8C64A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F21" xr:uid="{09DA59E2-D660-4205-9BDA-D6F8BD5435B1}">
       <formula1>"UF,PERSONAL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H20" xr:uid="{5A6C04F6-C6E3-4E26-8C34-95A9F129A7E6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H21" xr:uid="{04A31BE1-7BB2-420A-86EC-C0F87E1247D3}">
       <formula1>"Air Fare,Taxi/Train/Bus,Car Rental,Gas/Tolls,Parking,Hotel,Bkfst,Lunch,Dinner,Phone/Data,Computer,Other,Postage,Misc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1127,7 +1167,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CA12799-134C-4E20-B6DB-9BDA421E472F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDCA18B0-3343-4D3C-9612-04A6FAF91FC0}">
   <sheetPr>
     <tabColor rgb="FFF0E4D6"/>
   </sheetPr>
@@ -1139,107 +1179,107 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add return flight rebooking fare difference to New Orleans report
Return leg changed from MSY-STL-OMA to MSY-DAL-OMA (WN4419/WN1374);
$105.01 fare difference charged to Visa -2674 on 7/8/26.
</commit_message>
<xml_diff>
--- a/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
+++ b/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\Group-2\travel\trips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D579A71-AF67-47A4-9961-D169BBD03062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CA69DC9-BC81-4E50-B858-696BBDBFACF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{665F24CF-46C1-42D5-94C2-B96555D6B5FA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{CDA97ACB-82DD-4719-A63A-D2FA111D3D56}"/>
   </bookViews>
   <sheets>
     <sheet name="ER Detail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
   <si>
     <t>UNIFOCUS EXPENSE REPORT  |  New Orleans - InterContinental (HM Alpha)</t>
   </si>
@@ -109,6 +109,9 @@
   </si>
   <si>
     <t>Lunch</t>
+  </si>
+  <si>
+    <t>SW fare difference - return leg rebooked MSY-DAL-OMA (WN4419/WN1374) replacing MSY-STL-OMA, Visa -2674</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -324,10 +327,10 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -666,11 +669,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD4AD5B1-FA26-448F-B874-DC9BF431DEC5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E658A25-1786-426F-AB45-15C98E29E7F3}">
   <sheetPr>
     <tabColor rgb="FFB6752E"/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" customWidth="1"/>
@@ -854,24 +857,38 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="13"/>
+      <c r="A8" s="13">
+        <v>46212</v>
+      </c>
       <c r="B8" s="14" t="str">
-        <f>IF(A8="","",TEXT(A8,"ddd"))</f>
-        <v/>
-      </c>
-      <c r="C8" s="19"/>
+        <f>TEXT(A8,"ddd")</f>
+        <v>Thu</v>
+      </c>
+      <c r="C8" s="15">
+        <v>105.01</v>
+      </c>
       <c r="D8" s="16">
         <v>1</v>
       </c>
       <c r="E8" s="15">
         <f>C8*D8</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="20"/>
+        <v>105.01</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="7"/>
@@ -879,7 +896,7 @@
         <f>IF(A9="","",TEXT(A9,"ddd"))</f>
         <v/>
       </c>
-      <c r="C9" s="21"/>
+      <c r="C9" s="19"/>
       <c r="D9" s="10">
         <v>1</v>
       </c>
@@ -891,7 +908,7 @@
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
-      <c r="J9" s="22"/>
+      <c r="J9" s="20"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="13"/>
@@ -899,7 +916,7 @@
         <f>IF(A10="","",TEXT(A10,"ddd"))</f>
         <v/>
       </c>
-      <c r="C10" s="19"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="16">
         <v>1</v>
       </c>
@@ -911,7 +928,7 @@
       <c r="G10" s="17"/>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
-      <c r="J10" s="20"/>
+      <c r="J10" s="22"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="7"/>
@@ -919,7 +936,7 @@
         <f>IF(A11="","",TEXT(A11,"ddd"))</f>
         <v/>
       </c>
-      <c r="C11" s="21"/>
+      <c r="C11" s="19"/>
       <c r="D11" s="10">
         <v>1</v>
       </c>
@@ -931,7 +948,7 @@
       <c r="G11" s="11"/>
       <c r="H11" s="11"/>
       <c r="I11" s="11"/>
-      <c r="J11" s="22"/>
+      <c r="J11" s="20"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="13"/>
@@ -939,7 +956,7 @@
         <f>IF(A12="","",TEXT(A12,"ddd"))</f>
         <v/>
       </c>
-      <c r="C12" s="19"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="16">
         <v>1</v>
       </c>
@@ -951,7 +968,7 @@
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
-      <c r="J12" s="20"/>
+      <c r="J12" s="22"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="7"/>
@@ -959,7 +976,7 @@
         <f>IF(A13="","",TEXT(A13,"ddd"))</f>
         <v/>
       </c>
-      <c r="C13" s="21"/>
+      <c r="C13" s="19"/>
       <c r="D13" s="10">
         <v>1</v>
       </c>
@@ -971,7 +988,7 @@
       <c r="G13" s="11"/>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
-      <c r="J13" s="22"/>
+      <c r="J13" s="20"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="13"/>
@@ -979,7 +996,7 @@
         <f>IF(A14="","",TEXT(A14,"ddd"))</f>
         <v/>
       </c>
-      <c r="C14" s="19"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="16">
         <v>1</v>
       </c>
@@ -991,7 +1008,7 @@
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
-      <c r="J14" s="20"/>
+      <c r="J14" s="22"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="7"/>
@@ -999,7 +1016,7 @@
         <f>IF(A15="","",TEXT(A15,"ddd"))</f>
         <v/>
       </c>
-      <c r="C15" s="21"/>
+      <c r="C15" s="19"/>
       <c r="D15" s="10">
         <v>1</v>
       </c>
@@ -1011,7 +1028,7 @@
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
-      <c r="J15" s="22"/>
+      <c r="J15" s="20"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="13"/>
@@ -1019,7 +1036,7 @@
         <f>IF(A16="","",TEXT(A16,"ddd"))</f>
         <v/>
       </c>
-      <c r="C16" s="19"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="16">
         <v>1</v>
       </c>
@@ -1031,7 +1048,7 @@
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
-      <c r="J16" s="20"/>
+      <c r="J16" s="22"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="7"/>
@@ -1039,7 +1056,7 @@
         <f>IF(A17="","",TEXT(A17,"ddd"))</f>
         <v/>
       </c>
-      <c r="C17" s="21"/>
+      <c r="C17" s="19"/>
       <c r="D17" s="10">
         <v>1</v>
       </c>
@@ -1051,7 +1068,7 @@
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
-      <c r="J17" s="22"/>
+      <c r="J17" s="20"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="13"/>
@@ -1059,7 +1076,7 @@
         <f>IF(A18="","",TEXT(A18,"ddd"))</f>
         <v/>
       </c>
-      <c r="C18" s="19"/>
+      <c r="C18" s="21"/>
       <c r="D18" s="16">
         <v>1</v>
       </c>
@@ -1071,7 +1088,7 @@
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
-      <c r="J18" s="20"/>
+      <c r="J18" s="22"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="7"/>
@@ -1079,7 +1096,7 @@
         <f>IF(A19="","",TEXT(A19,"ddd"))</f>
         <v/>
       </c>
-      <c r="C19" s="21"/>
+      <c r="C19" s="19"/>
       <c r="D19" s="10">
         <v>1</v>
       </c>
@@ -1091,7 +1108,7 @@
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
-      <c r="J19" s="22"/>
+      <c r="J19" s="20"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="13"/>
@@ -1099,7 +1116,7 @@
         <f>IF(A20="","",TEXT(A20,"ddd"))</f>
         <v/>
       </c>
-      <c r="C20" s="19"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="16">
         <v>1</v>
       </c>
@@ -1111,7 +1128,7 @@
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="20"/>
+      <c r="J20" s="22"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="7"/>
@@ -1119,7 +1136,7 @@
         <f>IF(A21="","",TEXT(A21,"ddd"))</f>
         <v/>
       </c>
-      <c r="C21" s="21"/>
+      <c r="C21" s="19"/>
       <c r="D21" s="10">
         <v>1</v>
       </c>
@@ -1131,34 +1148,54 @@
       <c r="G21" s="11"/>
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
-      <c r="J21" s="22"/>
+      <c r="J21" s="20"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="E22" s="25">
-        <f>SUM(E5:E21)</f>
-        <v>892.47000000000014</v>
-      </c>
-      <c r="F22" s="23"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="23"/>
-      <c r="J22" s="23"/>
+      <c r="A22" s="13"/>
+      <c r="B22" s="14" t="str">
+        <f>IF(A22="","",TEXT(A22,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="C22" s="21"/>
+      <c r="D22" s="16">
+        <v>1</v>
+      </c>
+      <c r="E22" s="15">
+        <f>C22*D22</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="22"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="23"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="25">
+        <f>SUM(E5:E22)</f>
+        <v>997.48000000000013</v>
+      </c>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F21" xr:uid="{09DA59E2-D660-4205-9BDA-D6F8BD5435B1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F22" xr:uid="{09DF835E-AFBD-4910-8FBE-F191AB5F0788}">
       <formula1>"UF,PERSONAL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H21" xr:uid="{04A31BE1-7BB2-420A-86EC-C0F87E1247D3}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H22" xr:uid="{A57B424C-EFA7-45D9-B0E5-3A5A7528D208}">
       <formula1>"Air Fare,Taxi/Train/Bus,Car Rental,Gas/Tolls,Parking,Hotel,Bkfst,Lunch,Dinner,Phone/Data,Computer,Other,Postage,Misc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1167,7 +1204,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDCA18B0-3343-4D3C-9612-04A6FAF91FC0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CB19181-2CD5-4F48-98BD-8F2E666EE489}">
   <sheetPr>
     <tabColor rgb="FFF0E4D6"/>
   </sheetPr>
@@ -1179,107 +1216,107 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate New Orleans expense report Excel with two more meal receipts
Sazerac Bar (MSY, $20.12) and Moe's Southwest Grill (DFW, $25.61) were
added to the build script by another session; rebuilding the .xlsx to
match.
</commit_message>
<xml_diff>
--- a/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
+++ b/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\Group-2\travel\trips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CA69DC9-BC81-4E50-B858-696BBDBFACF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EBEAD46-A81F-4AE9-BF43-060B87073FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{CDA97ACB-82DD-4719-A63A-D2FA111D3D56}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{7CAB185F-10D5-42CD-9869-A2D82FAB803E}"/>
   </bookViews>
   <sheets>
     <sheet name="ER Detail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="49">
   <si>
     <t>UNIFOCUS EXPENSE REPORT  |  New Orleans - InterContinental (HM Alpha)</t>
   </si>
@@ -112,6 +112,15 @@
   </si>
   <si>
     <t>SW fare difference - return leg rebooked MSY-DAL-OMA (WN4419/WN1374) replacing MSY-STL-OMA, Visa -2674</t>
+  </si>
+  <si>
+    <t>Sazerac Bar, New Orleans Airport (MSY) - sweet chili glazed chicken sandwich, CC surcharge, tip</t>
+  </si>
+  <si>
+    <t>Moe's Southwest Grill, DFW Airport (return layover) - chicken burrito bowl, Coke Zero, cookie, tip</t>
+  </si>
+  <si>
+    <t>Dinner</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -669,11 +678,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E658A25-1786-426F-AB45-15C98E29E7F3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28E0F2BE-4055-40D8-9415-4139B9A0BF8C}">
   <sheetPr>
     <tabColor rgb="FFB6752E"/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" customWidth="1"/>
@@ -891,44 +900,72 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="7"/>
+      <c r="A9" s="7">
+        <v>46212</v>
+      </c>
       <c r="B9" s="8" t="str">
-        <f>IF(A9="","",TEXT(A9,"ddd"))</f>
-        <v/>
-      </c>
-      <c r="C9" s="19"/>
+        <f>TEXT(A9,"ddd")</f>
+        <v>Thu</v>
+      </c>
+      <c r="C9" s="9">
+        <v>20.12</v>
+      </c>
       <c r="D9" s="10">
         <v>1</v>
       </c>
       <c r="E9" s="9">
         <f>C9*D9</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="20"/>
+        <v>20.12</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="13"/>
+      <c r="A10" s="13">
+        <v>46212</v>
+      </c>
       <c r="B10" s="14" t="str">
-        <f>IF(A10="","",TEXT(A10,"ddd"))</f>
-        <v/>
-      </c>
-      <c r="C10" s="21"/>
+        <f>TEXT(A10,"ddd")</f>
+        <v>Thu</v>
+      </c>
+      <c r="C10" s="15">
+        <v>25.61</v>
+      </c>
       <c r="D10" s="16">
         <v>1</v>
       </c>
       <c r="E10" s="15">
         <f>C10*D10</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="22"/>
+        <v>25.61</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="18" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="7"/>
@@ -1171,31 +1208,71 @@
       <c r="J22" s="22"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="E23" s="25">
-        <f>SUM(E5:E22)</f>
-        <v>997.48000000000013</v>
-      </c>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="23"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="8" t="str">
+        <f>IF(A23="","",TEXT(A23,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="C23" s="19"/>
+      <c r="D23" s="10">
+        <v>1</v>
+      </c>
+      <c r="E23" s="9">
+        <f>C23*D23</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="20"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="13"/>
+      <c r="B24" s="14" t="str">
+        <f>IF(A24="","",TEXT(A24,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="C24" s="21"/>
+      <c r="D24" s="16">
+        <v>1</v>
+      </c>
+      <c r="E24" s="15">
+        <f>C24*D24</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="22"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="23"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25" s="25">
+        <f>SUM(E5:E24)</f>
+        <v>1043.21</v>
+      </c>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F22" xr:uid="{09DF835E-AFBD-4910-8FBE-F191AB5F0788}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F24" xr:uid="{C554593C-9E73-4037-9673-39282A60EF1C}">
       <formula1>"UF,PERSONAL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H22" xr:uid="{A57B424C-EFA7-45D9-B0E5-3A5A7528D208}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H24" xr:uid="{1ABF0753-CED2-45FD-8363-C2C7ADFF7E78}">
       <formula1>"Air Fare,Taxi/Train/Bus,Car Rental,Gas/Tolls,Parking,Hotel,Bkfst,Lunch,Dinner,Phone/Data,Computer,Other,Postage,Misc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1204,7 +1281,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CB19181-2CD5-4F48-98BD-8F2E666EE489}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E23F4829-3C03-4C28-8BAE-E0A4270869A3}">
   <sheetPr>
     <tabColor rgb="FFF0E4D6"/>
   </sheetPr>
@@ -1216,107 +1293,107 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Uber MSY receipt to NOLA expense report; log BTTR icons/plaza + benches call notes
- Add Uber MSY-to-hotel ride ($44.34) to New Orleans receipt log and expense report as Taxi/Train/Bus
- Save receipt PDF to travel/trips/receipts with standard naming
- Capture Larry Foster call notes: BTTR icons/plaza project (HGM/HDM contractor engagement), July 17 board meeting prep, benches/plaques decision

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
+++ b/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\Group-2\travel\trips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EBEAD46-A81F-4AE9-BF43-060B87073FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C655FB5F-049D-48D1-9341-164BD2697C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{7CAB185F-10D5-42CD-9869-A2D82FAB803E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{B80F1AF7-3B3C-4377-9F65-C4F92C971CAB}"/>
   </bookViews>
   <sheets>
     <sheet name="ER Detail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="51">
   <si>
     <t>UNIFOCUS EXPENSE REPORT  |  New Orleans - InterContinental (HM Alpha)</t>
   </si>
@@ -109,6 +109,12 @@
   </si>
   <si>
     <t>Lunch</t>
+  </si>
+  <si>
+    <t>Uber - MSY Airport to InterContinental New Orleans (444 St Charles Ave), 15.96 mi/22 min, driver Kathryn, Visa -0733 (FNBO Evergreen)</t>
+  </si>
+  <si>
+    <t>Taxi/Train/Bus</t>
   </si>
   <si>
     <t>SW fare difference - return leg rebooked MSY-DAL-OMA (WN4419/WN1374) replacing MSY-STL-OMA, Visa -2674</t>
@@ -336,10 +342,10 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -678,11 +684,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28E0F2BE-4055-40D8-9415-4139B9A0BF8C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7283BFB-0CED-49B1-8ED1-951BFA4737B0}">
   <sheetPr>
     <tabColor rgb="FFB6752E"/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" customWidth="1"/>
@@ -867,21 +873,21 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="13">
-        <v>46212</v>
+        <v>46209</v>
       </c>
       <c r="B8" s="14" t="str">
         <f>TEXT(A8,"ddd")</f>
-        <v>Thu</v>
+        <v>Mon</v>
       </c>
       <c r="C8" s="15">
-        <v>105.01</v>
+        <v>44.34</v>
       </c>
       <c r="D8" s="16">
         <v>1</v>
       </c>
       <c r="E8" s="15">
         <f>C8*D8</f>
-        <v>105.01</v>
+        <v>44.34</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>15</v>
@@ -890,7 +896,7 @@
         <v>23</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="I8" s="17" t="s">
         <v>18</v>
@@ -908,23 +914,23 @@
         <v>Thu</v>
       </c>
       <c r="C9" s="9">
-        <v>20.12</v>
+        <v>105.01</v>
       </c>
       <c r="D9" s="10">
         <v>1</v>
       </c>
       <c r="E9" s="9">
         <f>C9*D9</f>
-        <v>20.12</v>
+        <v>105.01</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>15</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I9" s="11" t="s">
         <v>18</v>
@@ -942,23 +948,23 @@
         <v>Thu</v>
       </c>
       <c r="C10" s="15">
-        <v>25.61</v>
+        <v>20.12</v>
       </c>
       <c r="D10" s="16">
         <v>1</v>
       </c>
       <c r="E10" s="15">
         <f>C10*D10</f>
-        <v>25.61</v>
+        <v>20.12</v>
       </c>
       <c r="F10" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="I10" s="17" t="s">
         <v>18</v>
@@ -968,24 +974,38 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="7"/>
+      <c r="A11" s="7">
+        <v>46212</v>
+      </c>
       <c r="B11" s="8" t="str">
-        <f>IF(A11="","",TEXT(A11,"ddd"))</f>
-        <v/>
-      </c>
-      <c r="C11" s="19"/>
+        <f>TEXT(A11,"ddd")</f>
+        <v>Thu</v>
+      </c>
+      <c r="C11" s="9">
+        <v>25.61</v>
+      </c>
       <c r="D11" s="10">
         <v>1</v>
       </c>
       <c r="E11" s="9">
         <f>C11*D11</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="20"/>
+        <v>25.61</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="13"/>
@@ -993,7 +1013,7 @@
         <f>IF(A12="","",TEXT(A12,"ddd"))</f>
         <v/>
       </c>
-      <c r="C12" s="21"/>
+      <c r="C12" s="19"/>
       <c r="D12" s="16">
         <v>1</v>
       </c>
@@ -1005,7 +1025,7 @@
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
-      <c r="J12" s="22"/>
+      <c r="J12" s="20"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="7"/>
@@ -1013,7 +1033,7 @@
         <f>IF(A13="","",TEXT(A13,"ddd"))</f>
         <v/>
       </c>
-      <c r="C13" s="19"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="10">
         <v>1</v>
       </c>
@@ -1025,7 +1045,7 @@
       <c r="G13" s="11"/>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
-      <c r="J13" s="20"/>
+      <c r="J13" s="22"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="13"/>
@@ -1033,7 +1053,7 @@
         <f>IF(A14="","",TEXT(A14,"ddd"))</f>
         <v/>
       </c>
-      <c r="C14" s="21"/>
+      <c r="C14" s="19"/>
       <c r="D14" s="16">
         <v>1</v>
       </c>
@@ -1045,7 +1065,7 @@
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
-      <c r="J14" s="22"/>
+      <c r="J14" s="20"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="7"/>
@@ -1053,7 +1073,7 @@
         <f>IF(A15="","",TEXT(A15,"ddd"))</f>
         <v/>
       </c>
-      <c r="C15" s="19"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="10">
         <v>1</v>
       </c>
@@ -1065,7 +1085,7 @@
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
-      <c r="J15" s="20"/>
+      <c r="J15" s="22"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="13"/>
@@ -1073,7 +1093,7 @@
         <f>IF(A16="","",TEXT(A16,"ddd"))</f>
         <v/>
       </c>
-      <c r="C16" s="21"/>
+      <c r="C16" s="19"/>
       <c r="D16" s="16">
         <v>1</v>
       </c>
@@ -1085,7 +1105,7 @@
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
-      <c r="J16" s="22"/>
+      <c r="J16" s="20"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="7"/>
@@ -1093,7 +1113,7 @@
         <f>IF(A17="","",TEXT(A17,"ddd"))</f>
         <v/>
       </c>
-      <c r="C17" s="19"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="10">
         <v>1</v>
       </c>
@@ -1105,7 +1125,7 @@
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
-      <c r="J17" s="20"/>
+      <c r="J17" s="22"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="13"/>
@@ -1113,7 +1133,7 @@
         <f>IF(A18="","",TEXT(A18,"ddd"))</f>
         <v/>
       </c>
-      <c r="C18" s="21"/>
+      <c r="C18" s="19"/>
       <c r="D18" s="16">
         <v>1</v>
       </c>
@@ -1125,7 +1145,7 @@
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
-      <c r="J18" s="22"/>
+      <c r="J18" s="20"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="7"/>
@@ -1133,7 +1153,7 @@
         <f>IF(A19="","",TEXT(A19,"ddd"))</f>
         <v/>
       </c>
-      <c r="C19" s="19"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="10">
         <v>1</v>
       </c>
@@ -1145,7 +1165,7 @@
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
-      <c r="J19" s="20"/>
+      <c r="J19" s="22"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="13"/>
@@ -1153,7 +1173,7 @@
         <f>IF(A20="","",TEXT(A20,"ddd"))</f>
         <v/>
       </c>
-      <c r="C20" s="21"/>
+      <c r="C20" s="19"/>
       <c r="D20" s="16">
         <v>1</v>
       </c>
@@ -1165,7 +1185,7 @@
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="22"/>
+      <c r="J20" s="20"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="7"/>
@@ -1173,7 +1193,7 @@
         <f>IF(A21="","",TEXT(A21,"ddd"))</f>
         <v/>
       </c>
-      <c r="C21" s="19"/>
+      <c r="C21" s="21"/>
       <c r="D21" s="10">
         <v>1</v>
       </c>
@@ -1185,7 +1205,7 @@
       <c r="G21" s="11"/>
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
-      <c r="J21" s="20"/>
+      <c r="J21" s="22"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="13"/>
@@ -1193,7 +1213,7 @@
         <f>IF(A22="","",TEXT(A22,"ddd"))</f>
         <v/>
       </c>
-      <c r="C22" s="21"/>
+      <c r="C22" s="19"/>
       <c r="D22" s="16">
         <v>1</v>
       </c>
@@ -1205,7 +1225,7 @@
       <c r="G22" s="17"/>
       <c r="H22" s="17"/>
       <c r="I22" s="17"/>
-      <c r="J22" s="22"/>
+      <c r="J22" s="20"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="7"/>
@@ -1213,7 +1233,7 @@
         <f>IF(A23="","",TEXT(A23,"ddd"))</f>
         <v/>
       </c>
-      <c r="C23" s="19"/>
+      <c r="C23" s="21"/>
       <c r="D23" s="10">
         <v>1</v>
       </c>
@@ -1225,7 +1245,7 @@
       <c r="G23" s="11"/>
       <c r="H23" s="11"/>
       <c r="I23" s="11"/>
-      <c r="J23" s="20"/>
+      <c r="J23" s="22"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="13"/>
@@ -1233,7 +1253,7 @@
         <f>IF(A24="","",TEXT(A24,"ddd"))</f>
         <v/>
       </c>
-      <c r="C24" s="21"/>
+      <c r="C24" s="19"/>
       <c r="D24" s="16">
         <v>1</v>
       </c>
@@ -1245,34 +1265,54 @@
       <c r="G24" s="17"/>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
-      <c r="J24" s="22"/>
+      <c r="J24" s="20"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="E25" s="25">
-        <f>SUM(E5:E24)</f>
-        <v>1043.21</v>
-      </c>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="8" t="str">
+        <f>IF(A25="","",TEXT(A25,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="C25" s="21"/>
+      <c r="D25" s="10">
+        <v>1</v>
+      </c>
+      <c r="E25" s="9">
+        <f>C25*D25</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="22"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="23"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" s="25">
+        <f>SUM(E5:E25)</f>
+        <v>1087.55</v>
+      </c>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F24" xr:uid="{C554593C-9E73-4037-9673-39282A60EF1C}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F25" xr:uid="{396E95A5-03E4-4AD5-8568-8F67AE50E540}">
       <formula1>"UF,PERSONAL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H24" xr:uid="{1ABF0753-CED2-45FD-8363-C2C7ADFF7E78}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H25" xr:uid="{7957B837-EF51-4766-8890-18157FB106E9}">
       <formula1>"Air Fare,Taxi/Train/Bus,Car Rental,Gas/Tolls,Parking,Hotel,Bkfst,Lunch,Dinner,Phone/Data,Computer,Other,Postage,Misc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1281,7 +1321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E23F4829-3C03-4C28-8BAE-E0A4270869A3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F350FB1-1F14-4920-9536-9B3CC3207A36}">
   <sheetPr>
     <tabColor rgb="FFF0E4D6"/>
   </sheetPr>
@@ -1293,107 +1333,107 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Summary tab to New Orleans expense report, matching Nashville/Pensacola format
Category and payment-type breakdown, plus open items, so all three trip
reports now share the same front-page summary style.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
+++ b/travel/trips/2026-07-06_2026-07-09_new-orleans-expense-report.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\Group-2\travel\trips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C655FB5F-049D-48D1-9341-164BD2697C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFC923CE-3559-40A0-A3A4-853879197AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{B80F1AF7-3B3C-4377-9F65-C4F92C971CAB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{64B2C944-0F93-48FC-AE4E-A3588B2B95AE}"/>
   </bookViews>
   <sheets>
-    <sheet name="ER Detail" sheetId="1" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="2" r:id="rId1"/>
+    <sheet name="ER Detail" sheetId="1" r:id="rId2"/>
+    <sheet name="Notes" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="79">
   <si>
     <t>UNIFOCUS EXPENSE REPORT  |  New Orleans - InterContinental (HM Alpha)</t>
   </si>
@@ -130,6 +131,90 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>NEW ORLEANS TRIP EXPENSE REPORT  -  JULY 6 to JULY 9, 2026</t>
+  </si>
+  <si>
+    <t>Traveler</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>HM Alpha training - InterContinental New Orleans (billable to Unifocus)</t>
+  </si>
+  <si>
+    <t>Dates</t>
+  </si>
+  <si>
+    <t>July 6 - July 9, 2026 (4 days)</t>
+  </si>
+  <si>
+    <t>Property</t>
+  </si>
+  <si>
+    <t>InterContinental New Orleans</t>
+  </si>
+  <si>
+    <t>Compiled</t>
+  </si>
+  <si>
+    <t>July 10, 2026</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Hotel comped by property. Trip reopened 7/10/26 to add Uber receipt found after close-out.</t>
+  </si>
+  <si>
+    <t>SUMMARY BY CATEGORY</t>
+  </si>
+  <si>
+    <t># Items</t>
+  </si>
+  <si>
+    <t>TOTAL REIMBURSABLE</t>
+  </si>
+  <si>
+    <t>SUMMARY BY PAYMENT TYPE</t>
+  </si>
+  <si>
+    <t>Payment Type</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>-2674</t>
+  </si>
+  <si>
+    <t>VISA SW Rapid Rewards+ (flight base + fare diff + Moe's DFW)</t>
+  </si>
+  <si>
+    <t>SW Credit</t>
+  </si>
+  <si>
+    <t>Southwest Flight Credit</t>
+  </si>
+  <si>
+    <t>Chase VISA</t>
+  </si>
+  <si>
+    <t>Chase VISA (Denver + Sazerac Bar lunches)</t>
+  </si>
+  <si>
+    <t>-0733</t>
+  </si>
+  <si>
+    <t>VISA Personal / FNBO Evergreen (Uber MSY)</t>
+  </si>
+  <si>
+    <t>OPEN ITEMS BEFORE SUBMISSION</t>
+  </si>
+  <si>
+    <t>Trip closed 7/10/26 - all known charges (flights, meals, Uber) reflected above.</t>
   </si>
   <si>
     <t>UNIFOCUS ER QUICK REFERENCE (from ER Cheat Sheet.pdf, dated 5/10/2021 - verify still current with Ralph if in doubt)</t>
@@ -202,7 +287,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,8 +319,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -272,6 +365,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -300,7 +405,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="36">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -350,6 +456,27 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -684,7 +811,280 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7283BFB-0CED-49B1-8ED1-951BFA4737B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17AE6FCC-49BD-4946-9E46-30278226B5CB}">
+  <sheetPr>
+    <tabColor rgb="FF64381F"/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.6328125" customWidth="1"/>
+    <col min="2" max="2" width="28.6328125" customWidth="1"/>
+    <col min="3" max="3" width="14.6328125" customWidth="1"/>
+    <col min="4" max="5" width="12.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="10">
+        <v>966.4</v>
+      </c>
+      <c r="C11" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="32">
+        <v>51.2</v>
+      </c>
+      <c r="C12" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="10">
+        <v>25.61</v>
+      </c>
+      <c r="C13" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="32">
+        <v>44.34</v>
+      </c>
+      <c r="C14" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="26">
+        <f>SUM(B11:B14)</f>
+        <v>1087.55</v>
+      </c>
+      <c r="C15" s="24"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="10">
+        <v>675.81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="32">
+        <v>316.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="10">
+        <v>51.2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="32">
+        <v>44.34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="24"/>
+      <c r="C23" s="26">
+        <f>SUM(C19:C22)</f>
+        <v>1087.55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BF7810D-B497-485E-AA46-8F47E5EEC762}">
   <sheetPr>
     <tabColor rgb="FFB6752E"/>
   </sheetPr>
@@ -704,615 +1104,615 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5">
         <v>46209</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="5">
         <v>46212</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="7">
+      <c r="A5" s="8">
         <v>46209</v>
       </c>
-      <c r="B5" s="8" t="str">
+      <c r="B5" s="9" t="str">
         <f>TEXT(A5,"ddd")</f>
         <v>Mon</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>545.19000000000005</v>
       </c>
-      <c r="D5" s="10">
-        <v>1</v>
-      </c>
-      <c r="E5" s="9">
+      <c r="D5" s="11">
+        <v>1</v>
+      </c>
+      <c r="E5" s="10">
         <f>C5*D5</f>
         <v>545.19000000000005</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="12" t="s">
+      <c r="J5" s="13" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="13">
+      <c r="A6" s="14">
         <v>46209</v>
       </c>
-      <c r="B6" s="14" t="str">
+      <c r="B6" s="15" t="str">
         <f>TEXT(A6,"ddd")</f>
         <v>Mon</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="16">
         <v>316.2</v>
       </c>
-      <c r="D6" s="16">
-        <v>1</v>
-      </c>
-      <c r="E6" s="15">
+      <c r="D6" s="17">
+        <v>1</v>
+      </c>
+      <c r="E6" s="16">
         <f>C6*D6</f>
         <v>316.2</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="17" t="s">
+      <c r="I6" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="18" t="s">
+      <c r="J6" s="19" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="7">
+      <c r="A7" s="8">
         <v>46209</v>
       </c>
-      <c r="B7" s="8" t="str">
+      <c r="B7" s="9" t="str">
         <f>TEXT(A7,"ddd")</f>
         <v>Mon</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>31.08</v>
       </c>
-      <c r="D7" s="10">
-        <v>1</v>
-      </c>
-      <c r="E7" s="9">
+      <c r="D7" s="11">
+        <v>1</v>
+      </c>
+      <c r="E7" s="10">
         <f>C7*D7</f>
         <v>31.08</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="12" t="s">
+      <c r="J7" s="13" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="13">
+      <c r="A8" s="14">
         <v>46209</v>
       </c>
-      <c r="B8" s="14" t="str">
+      <c r="B8" s="15" t="str">
         <f>TEXT(A8,"ddd")</f>
         <v>Mon</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>44.34</v>
       </c>
-      <c r="D8" s="16">
-        <v>1</v>
-      </c>
-      <c r="E8" s="15">
+      <c r="D8" s="17">
+        <v>1</v>
+      </c>
+      <c r="E8" s="16">
         <f>C8*D8</f>
         <v>44.34</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="17" t="s">
+      <c r="I8" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="18" t="s">
+      <c r="J8" s="19" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="7">
+      <c r="A9" s="8">
         <v>46212</v>
       </c>
-      <c r="B9" s="8" t="str">
+      <c r="B9" s="9" t="str">
         <f>TEXT(A9,"ddd")</f>
         <v>Thu</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="10">
         <v>105.01</v>
       </c>
-      <c r="D9" s="10">
-        <v>1</v>
-      </c>
-      <c r="E9" s="9">
+      <c r="D9" s="11">
+        <v>1</v>
+      </c>
+      <c r="E9" s="10">
         <f>C9*D9</f>
         <v>105.01</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I9" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="12" t="s">
+      <c r="J9" s="13" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="13">
+      <c r="A10" s="14">
         <v>46212</v>
       </c>
-      <c r="B10" s="14" t="str">
+      <c r="B10" s="15" t="str">
         <f>TEXT(A10,"ddd")</f>
         <v>Thu</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>20.12</v>
       </c>
-      <c r="D10" s="16">
-        <v>1</v>
-      </c>
-      <c r="E10" s="15">
+      <c r="D10" s="17">
+        <v>1</v>
+      </c>
+      <c r="E10" s="16">
         <f>C10*D10</f>
         <v>20.12</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="17" t="s">
+      <c r="G10" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="I10" s="17" t="s">
+      <c r="I10" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="J10" s="18" t="s">
+      <c r="J10" s="19" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="7">
+      <c r="A11" s="8">
         <v>46212</v>
       </c>
-      <c r="B11" s="8" t="str">
+      <c r="B11" s="9" t="str">
         <f>TEXT(A11,"ddd")</f>
         <v>Thu</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>25.61</v>
       </c>
-      <c r="D11" s="10">
-        <v>1</v>
-      </c>
-      <c r="E11" s="9">
+      <c r="D11" s="11">
+        <v>1</v>
+      </c>
+      <c r="E11" s="10">
         <f>C11*D11</f>
         <v>25.61</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="I11" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="12" t="s">
+      <c r="J11" s="13" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14" t="str">
+      <c r="A12" s="14"/>
+      <c r="B12" s="15" t="str">
         <f>IF(A12="","",TEXT(A12,"ddd"))</f>
         <v/>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="16">
-        <v>1</v>
-      </c>
-      <c r="E12" s="15">
+      <c r="C12" s="20"/>
+      <c r="D12" s="17">
+        <v>1</v>
+      </c>
+      <c r="E12" s="16">
         <f>C12*D12</f>
         <v>0</v>
       </c>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="20"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="21"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8" t="str">
+      <c r="A13" s="8"/>
+      <c r="B13" s="9" t="str">
         <f>IF(A13="","",TEXT(A13,"ddd"))</f>
         <v/>
       </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="10">
-        <v>1</v>
-      </c>
-      <c r="E13" s="9">
+      <c r="C13" s="22"/>
+      <c r="D13" s="11">
+        <v>1</v>
+      </c>
+      <c r="E13" s="10">
         <f>C13*D13</f>
         <v>0</v>
       </c>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="22"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="23"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14" t="str">
+      <c r="A14" s="14"/>
+      <c r="B14" s="15" t="str">
         <f>IF(A14="","",TEXT(A14,"ddd"))</f>
         <v/>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="16">
-        <v>1</v>
-      </c>
-      <c r="E14" s="15">
+      <c r="C14" s="20"/>
+      <c r="D14" s="17">
+        <v>1</v>
+      </c>
+      <c r="E14" s="16">
         <f>C14*D14</f>
         <v>0</v>
       </c>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="20"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="21"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8" t="str">
+      <c r="A15" s="8"/>
+      <c r="B15" s="9" t="str">
         <f>IF(A15="","",TEXT(A15,"ddd"))</f>
         <v/>
       </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="10">
-        <v>1</v>
-      </c>
-      <c r="E15" s="9">
+      <c r="C15" s="22"/>
+      <c r="D15" s="11">
+        <v>1</v>
+      </c>
+      <c r="E15" s="10">
         <f>C15*D15</f>
         <v>0</v>
       </c>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="22"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="23"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14" t="str">
+      <c r="A16" s="14"/>
+      <c r="B16" s="15" t="str">
         <f>IF(A16="","",TEXT(A16,"ddd"))</f>
         <v/>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="16">
-        <v>1</v>
-      </c>
-      <c r="E16" s="15">
+      <c r="C16" s="20"/>
+      <c r="D16" s="17">
+        <v>1</v>
+      </c>
+      <c r="E16" s="16">
         <f>C16*D16</f>
         <v>0</v>
       </c>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="20"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="21"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="7"/>
-      <c r="B17" s="8" t="str">
+      <c r="A17" s="8"/>
+      <c r="B17" s="9" t="str">
         <f>IF(A17="","",TEXT(A17,"ddd"))</f>
         <v/>
       </c>
-      <c r="C17" s="21"/>
-      <c r="D17" s="10">
-        <v>1</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="C17" s="22"/>
+      <c r="D17" s="11">
+        <v>1</v>
+      </c>
+      <c r="E17" s="10">
         <f>C17*D17</f>
         <v>0</v>
       </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="22"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="23"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14" t="str">
+      <c r="A18" s="14"/>
+      <c r="B18" s="15" t="str">
         <f>IF(A18="","",TEXT(A18,"ddd"))</f>
         <v/>
       </c>
-      <c r="C18" s="19"/>
-      <c r="D18" s="16">
-        <v>1</v>
-      </c>
-      <c r="E18" s="15">
+      <c r="C18" s="20"/>
+      <c r="D18" s="17">
+        <v>1</v>
+      </c>
+      <c r="E18" s="16">
         <f>C18*D18</f>
         <v>0</v>
       </c>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="20"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="21"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="7"/>
-      <c r="B19" s="8" t="str">
+      <c r="A19" s="8"/>
+      <c r="B19" s="9" t="str">
         <f>IF(A19="","",TEXT(A19,"ddd"))</f>
         <v/>
       </c>
-      <c r="C19" s="21"/>
-      <c r="D19" s="10">
-        <v>1</v>
-      </c>
-      <c r="E19" s="9">
+      <c r="C19" s="22"/>
+      <c r="D19" s="11">
+        <v>1</v>
+      </c>
+      <c r="E19" s="10">
         <f>C19*D19</f>
         <v>0</v>
       </c>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="22"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="23"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14" t="str">
+      <c r="A20" s="14"/>
+      <c r="B20" s="15" t="str">
         <f>IF(A20="","",TEXT(A20,"ddd"))</f>
         <v/>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="16">
-        <v>1</v>
-      </c>
-      <c r="E20" s="15">
+      <c r="C20" s="20"/>
+      <c r="D20" s="17">
+        <v>1</v>
+      </c>
+      <c r="E20" s="16">
         <f>C20*D20</f>
         <v>0</v>
       </c>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="20"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="21"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="7"/>
-      <c r="B21" s="8" t="str">
+      <c r="A21" s="8"/>
+      <c r="B21" s="9" t="str">
         <f>IF(A21="","",TEXT(A21,"ddd"))</f>
         <v/>
       </c>
-      <c r="C21" s="21"/>
-      <c r="D21" s="10">
-        <v>1</v>
-      </c>
-      <c r="E21" s="9">
+      <c r="C21" s="22"/>
+      <c r="D21" s="11">
+        <v>1</v>
+      </c>
+      <c r="E21" s="10">
         <f>C21*D21</f>
         <v>0</v>
       </c>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="22"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="23"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14" t="str">
+      <c r="A22" s="14"/>
+      <c r="B22" s="15" t="str">
         <f>IF(A22="","",TEXT(A22,"ddd"))</f>
         <v/>
       </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="16">
-        <v>1</v>
-      </c>
-      <c r="E22" s="15">
+      <c r="C22" s="20"/>
+      <c r="D22" s="17">
+        <v>1</v>
+      </c>
+      <c r="E22" s="16">
         <f>C22*D22</f>
         <v>0</v>
       </c>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="20"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="21"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="7"/>
-      <c r="B23" s="8" t="str">
+      <c r="A23" s="8"/>
+      <c r="B23" s="9" t="str">
         <f>IF(A23="","",TEXT(A23,"ddd"))</f>
         <v/>
       </c>
-      <c r="C23" s="21"/>
-      <c r="D23" s="10">
-        <v>1</v>
-      </c>
-      <c r="E23" s="9">
+      <c r="C23" s="22"/>
+      <c r="D23" s="11">
+        <v>1</v>
+      </c>
+      <c r="E23" s="10">
         <f>C23*D23</f>
         <v>0</v>
       </c>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="22"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="23"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14" t="str">
+      <c r="A24" s="14"/>
+      <c r="B24" s="15" t="str">
         <f>IF(A24="","",TEXT(A24,"ddd"))</f>
         <v/>
       </c>
-      <c r="C24" s="19"/>
-      <c r="D24" s="16">
-        <v>1</v>
-      </c>
-      <c r="E24" s="15">
+      <c r="C24" s="20"/>
+      <c r="D24" s="17">
+        <v>1</v>
+      </c>
+      <c r="E24" s="16">
         <f>C24*D24</f>
         <v>0</v>
       </c>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="20"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="21"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="7"/>
-      <c r="B25" s="8" t="str">
+      <c r="A25" s="8"/>
+      <c r="B25" s="9" t="str">
         <f>IF(A25="","",TEXT(A25,"ddd"))</f>
         <v/>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="10">
-        <v>1</v>
-      </c>
-      <c r="E25" s="9">
+      <c r="C25" s="22"/>
+      <c r="D25" s="11">
+        <v>1</v>
+      </c>
+      <c r="E25" s="10">
         <f>C25*D25</f>
         <v>0</v>
       </c>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="22"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="23"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="24" t="s">
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="25">
+      <c r="E26" s="26">
         <f>SUM(E5:E25)</f>
         <v>1087.55</v>
       </c>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="23"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F25" xr:uid="{396E95A5-03E4-4AD5-8568-8F67AE50E540}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F25" xr:uid="{657DA54A-00F8-451D-8919-113B6B7AAFDB}">
       <formula1>"UF,PERSONAL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H25" xr:uid="{7957B837-EF51-4766-8890-18157FB106E9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H25" xr:uid="{E58F13A9-8EAD-4811-9EF4-D06A7780CC7F}">
       <formula1>"Air Fare,Taxi/Train/Bus,Car Rental,Gas/Tolls,Parking,Hotel,Bkfst,Lunch,Dinner,Phone/Data,Computer,Other,Postage,Misc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1320,8 +1720,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F350FB1-1F14-4920-9536-9B3CC3207A36}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5841473F-8F48-4220-BB23-29960504867E}">
   <sheetPr>
     <tabColor rgb="FFF0E4D6"/>
   </sheetPr>
@@ -1332,108 +1732,108 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
-        <v>30</v>
+      <c r="A1" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>